<commit_message>
Dyamic flow in load ats and generate ats
</commit_message>
<xml_diff>
--- a/src/test/resources/files/updatedbr.xlsx
+++ b/src/test/resources/files/updatedbr.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\API-Automation\src\test\resources\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -153,10 +153,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -512,11 +515,11 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" ht="84">
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
@@ -525,11 +528,11 @@
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" ht="84">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">

</xml_diff>